<commit_message>
add tab with titles in export
</commit_message>
<xml_diff>
--- a/exports/WIC2026_Programme_Publish.xlsx
+++ b/exports/WIC2026_Programme_Publish.xlsx
@@ -13,19 +13,20 @@
     <sheet name="Day 3" sheetId="4" r:id="rId4"/>
     <sheet name="Session Directory" sheetId="5" r:id="rId5"/>
     <sheet name="Paper Index" sheetId="6" r:id="rId6"/>
-    <sheet name="Issues" sheetId="7" r:id="rId7"/>
+    <sheet name="Title Presenter Index" sheetId="7" r:id="rId7"/>
+    <sheet name="Issues" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2565" uniqueCount="836">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3109" uniqueCount="1344">
   <si>
     <t>World Inequality Conference 2026</t>
   </si>
   <si>
-    <t>Generated: 2026-04-23 17:52</t>
+    <t>Generated: 2026-04-24 14:39</t>
   </si>
   <si>
     <t>This programme covers parallel sessions only. For plenary sessions, see the plenary sessions programme.</t>
@@ -21216,6 +21217,1632 @@
     <t>zxRbM51</t>
   </si>
   <si>
+    <t>Presentation Title</t>
+  </si>
+  <si>
+    <t>Presenter Name</t>
+  </si>
+  <si>
+    <t>The Global Democratic Deficit: Institutional Asymetries and the Provision of Global Public Goods</t>
+  </si>
+  <si>
+    <t>Paula Druschke &amp; Gaston Nievas</t>
+  </si>
+  <si>
+    <t>Market power, growth and wealth inequality</t>
+  </si>
+  <si>
+    <t>Giammario Impullitti</t>
+  </si>
+  <si>
+    <t>Gender and intergenerational mobility: unequal economic outcomes between siblings</t>
+  </si>
+  <si>
+    <t>Martin Leites</t>
+  </si>
+  <si>
+    <t>Private Capital Markets and Inequality</t>
+  </si>
+  <si>
+    <t>Ararat Gocmen - Clara Martinez-Toledano</t>
+  </si>
+  <si>
+    <t>Non-Stationary Wealth Dynamics and Taxation in the U.S. With an Application to the Racial Gap</t>
+  </si>
+  <si>
+    <t>Alberto Bisin</t>
+  </si>
+  <si>
+    <t>The last IMF loan to Argentina: Were gender clauses effective in protecting women?</t>
+  </si>
+  <si>
+    <t>Mercedes DAlessandro</t>
+  </si>
+  <si>
+    <t>Left Behind? West-East German Disparities in the Cost of Job Loss</t>
+  </si>
+  <si>
+    <t>César Barreto</t>
+  </si>
+  <si>
+    <t>Public Works Program, Labor Supply, and Monopsony</t>
+  </si>
+  <si>
+    <t>Tsenguunjav Byambasuren</t>
+  </si>
+  <si>
+    <t>Willing but Unable: Social Norms and Costs of Female Hiring in Pakistan</t>
+  </si>
+  <si>
+    <t>Zunia Saif Tirmazee</t>
+  </si>
+  <si>
+    <t>Has Experience Made Me Rich? Analysis of the U.S. Gender Wealth Gap</t>
+  </si>
+  <si>
+    <t>Jesse Bricker</t>
+  </si>
+  <si>
+    <t>Personal Holding Companies, Tax Progressivity, and Inequality</t>
+  </si>
+  <si>
+    <t>Gabriel Zucman</t>
+  </si>
+  <si>
+    <t>Shift or Share? Profit Shifting and Implications for Workers Profit-Sharing</t>
+  </si>
+  <si>
+    <t>Laure Heidmann</t>
+  </si>
+  <si>
+    <t>Lifting Each Other Up: How Cooperative Firms Foster Local Development</t>
+  </si>
+  <si>
+    <t>Guillermo Woo-Mora</t>
+  </si>
+  <si>
+    <t>Using trusts in the UK: income, wealth and beneficiaries</t>
+  </si>
+  <si>
+    <t>Sanaya Mahajan</t>
+  </si>
+  <si>
+    <t>Economic Elites and Wealth Concentration Cross-Nationally, 1996-2025</t>
+  </si>
+  <si>
+    <t>Wesley Stubenbord</t>
+  </si>
+  <si>
+    <t>Inequality and Redistribution in Switzerland: Evidence from Distributional National Accounts</t>
+  </si>
+  <si>
+    <t>Julian Koller</t>
+  </si>
+  <si>
+    <t>Product Market Monopolies and Labor Market Monopsonies</t>
+  </si>
+  <si>
+    <t>Massimiliano Cali</t>
+  </si>
+  <si>
+    <t>Line drawing: can poverty measurement inform the methodology for a social indicator of extreme wealth?</t>
+  </si>
+  <si>
+    <t>Tania Burchardt</t>
+  </si>
+  <si>
+    <t>The Race Between Technology and Sobriety: Distributional Pathways to Planetary Sustainability</t>
+  </si>
+  <si>
+    <t>Marco Ranaldi</t>
+  </si>
+  <si>
+    <t>Glorious for whom? Income inequality in the Netherlands during les Trente Glorieuses</t>
+  </si>
+  <si>
+    <t>Sarah Kuypers</t>
+  </si>
+  <si>
+    <t>The Western Exception: Declining Inequality and Persistent Political Cleavages in Portugal</t>
+  </si>
+  <si>
+    <t>Carlos Oliveira</t>
+  </si>
+  <si>
+    <t>Weather Shocks and Manufactured Exports from Sub-Saharan Africa: How Economic Freedom and Institutional Quality Shape Resilience</t>
+  </si>
+  <si>
+    <t>Dr. Andrew Ojede</t>
+  </si>
+  <si>
+    <t>Progress and Persistence: Race and Intergenerational Educational Mobility in South Africa</t>
+  </si>
+  <si>
+    <t>Timothy Köhler</t>
+  </si>
+  <si>
+    <t>Natural resources and gender (in)equality in education in Africa</t>
+  </si>
+  <si>
+    <t>Idrissa Ouedraogo</t>
+  </si>
+  <si>
+    <t>Measuring long-run wealth inequality: Empirical results for Norway 1912-2019</t>
+  </si>
+  <si>
+    <t>Jørgen Modalsli</t>
+  </si>
+  <si>
+    <t>Real estate wealth inequality and exposure to natural disasters</t>
+  </si>
+  <si>
+    <t>Thomas Bezy</t>
+  </si>
+  <si>
+    <t>Transaction Taxes and Housing Inequality: Evidence from the UK Stamp Duty Holiday</t>
+  </si>
+  <si>
+    <t>Yonatan Berman</t>
+  </si>
+  <si>
+    <t>Do Public Goods Actually Reduce Inequality?</t>
+  </si>
+  <si>
+    <t>Micael Castanheira</t>
+  </si>
+  <si>
+    <t>The Negative Impact of Colonization on the Local Population: Evidence from Morocco</t>
+  </si>
+  <si>
+    <t>Ariane Salem</t>
+  </si>
+  <si>
+    <t>Global Justice Pathways for Ten Billion: Inequality, Risk Sharing and Planetary Boundaries to 2100</t>
+  </si>
+  <si>
+    <t>Joel Naoki Ernesto Christoph</t>
+  </si>
+  <si>
+    <t>Who benefits from land take? Inequality, property ownership and the ecological debt of artificialization in France</t>
+  </si>
+  <si>
+    <t>Eulalie Saïsset</t>
+  </si>
+  <si>
+    <t>Portfolio Allocation and Housing Markets</t>
+  </si>
+  <si>
+    <t>Rémi Lei</t>
+  </si>
+  <si>
+    <t>Stayin’ Elite: Wealth, Multigenerational Persistence, and Political Power Among the US Hyperwealthy, 1875-1950</t>
+  </si>
+  <si>
+    <t>Julian Costas-Fernandez</t>
+  </si>
+  <si>
+    <t>A Scrooge McDuck Theory of Wealth Dynamics</t>
+  </si>
+  <si>
+    <t>Valentin Marchal</t>
+  </si>
+  <si>
+    <t>Class Mobility in the Era of Rising Inequality: A Synthetic Dynasty Analysis</t>
+  </si>
+  <si>
+    <t>Kristina Butaeva</t>
+  </si>
+  <si>
+    <t>Do Billionaires Pay Taxes?</t>
+  </si>
+  <si>
+    <t>Clément Malgouyres</t>
+  </si>
+  <si>
+    <t>Source Decomposition of Inequality Revisited</t>
+  </si>
+  <si>
+    <t>Vesa-Matti Heikkuri</t>
+  </si>
+  <si>
+    <t>Top x%, Income Inequality and Social Welfare</t>
+  </si>
+  <si>
+    <t>Antoine Germain</t>
+  </si>
+  <si>
+    <t>The Effects of Minimum Wage Increases on Poverty and Food Hardship</t>
+  </si>
+  <si>
+    <t>Lukas Lehner</t>
+  </si>
+  <si>
+    <t>Extreme Income Inequality in Ecuador - Dollarization, Commodity Price Boom, and Citizen Revolution</t>
+  </si>
+  <si>
+    <t>Markus Nabernegg</t>
+  </si>
+  <si>
+    <t>Political inclusion and economic inequality in the long run: Central-Northern Italy, 1500-1800</t>
+  </si>
+  <si>
+    <t>Giulio Ongaro</t>
+  </si>
+  <si>
+    <t>How Much Tax Do US Billionaires Pay? Evidence from Administrative Data</t>
+  </si>
+  <si>
+    <t>Emmanuel Saez</t>
+  </si>
+  <si>
+    <t>Technological Change and Racial Disparities</t>
+  </si>
+  <si>
+    <t>Vittoria Dicandia</t>
+  </si>
+  <si>
+    <t>When Bankers Become Informants: Behavioral Effects of Automatic Exchange of Information</t>
+  </si>
+  <si>
+    <t>Jeanne Bomare</t>
+  </si>
+  <si>
+    <t>Income &amp; Wealth in WW2-France: A Macroeconomic &amp; Fiscal Overview</t>
+  </si>
+  <si>
+    <t>Pierre Brassac</t>
+  </si>
+  <si>
+    <t>Death and Taxes: Inheritance Tax Planning and Unexpected Mortality</t>
+  </si>
+  <si>
+    <t>Ignacio Orueta</t>
+  </si>
+  <si>
+    <t>Scale-dependent returns and the interest rate</t>
+  </si>
+  <si>
+    <t>Mojtaba Hayati</t>
+  </si>
+  <si>
+    <t>Time for Development</t>
+  </si>
+  <si>
+    <t>Jihoon Min</t>
+  </si>
+  <si>
+    <t>Wealth Mobility in the United States: Empirical Evidence from the PSID</t>
+  </si>
+  <si>
+    <t>Christophe Van Langenhove</t>
+  </si>
+  <si>
+    <t>Identification of Child Penalties</t>
+  </si>
+  <si>
+    <t>Dor Leventer</t>
+  </si>
+  <si>
+    <t>Extreme Inequality and Economic Growth</t>
+  </si>
+  <si>
+    <t>Suranjana Kundu</t>
+  </si>
+  <si>
+    <t>From fragile careers to inadequate pensions: a cohort comparison of career dynamics in Italy</t>
+  </si>
+  <si>
+    <t>Francesca Subioli</t>
+  </si>
+  <si>
+    <t>The Return of Inheritance</t>
+  </si>
+  <si>
+    <t>Demetrio Guzzardi</t>
+  </si>
+  <si>
+    <t>Measuring Global Inequality: How accounting for inequality within the household affects the global profile</t>
+  </si>
+  <si>
+    <t>Samuel Kofi Tetteh-Baah</t>
+  </si>
+  <si>
+    <t>Global Inequality by 2050: The Role of Redistribution and Climate Change</t>
+  </si>
+  <si>
+    <t>Cornelia Mohren</t>
+  </si>
+  <si>
+    <t>Poverty and Mobility in the Time of Synthetic Panels: Evidence from Argentina (2003–2023)</t>
+  </si>
+  <si>
+    <t>Nicolas Larrea Avila</t>
+  </si>
+  <si>
+    <t>Capital and Labor Income Mobility</t>
+  </si>
+  <si>
+    <t>Roberto Iacono</t>
+  </si>
+  <si>
+    <t>National Service and the Great Leveling: New evidence on midcentury American inequality</t>
+  </si>
+  <si>
+    <t>Matthew Fisher-Post</t>
+  </si>
+  <si>
+    <t>The double glass ceiling: Female top incomes and the role of capital</t>
+  </si>
+  <si>
+    <t>Lotte Maaßen</t>
+  </si>
+  <si>
+    <t>Understanding Survey Income Errors Using Linked Administrative Data</t>
+  </si>
+  <si>
+    <t>Dongwoong Seo</t>
+  </si>
+  <si>
+    <t>Solving science conundrums in the climate-nature-equity polycrisis: The need for transformative, socially just, climate and biodiversity scenarios</t>
+  </si>
+  <si>
+    <t>Laura Pereira</t>
+  </si>
+  <si>
+    <t>The equity and efficiency of carbon taxation: a multi-model, multi-country analysis</t>
+  </si>
+  <si>
+    <t>Julien Lefevre</t>
+  </si>
+  <si>
+    <t>Billionaires’ emissions and climate finance: the case for a carbon wealth tax</t>
+  </si>
+  <si>
+    <t>Elisa Palagi</t>
+  </si>
+  <si>
+    <t>What do we know about wealth inequality in Brazil?</t>
+  </si>
+  <si>
+    <t>Pedro Fandiño</t>
+  </si>
+  <si>
+    <t>Global Wealth Accumulation and Ownership Patterns, 1800-2025</t>
+  </si>
+  <si>
+    <t>Alice Sodano</t>
+  </si>
+  <si>
+    <t>A Carbon Wealth Tax: Modelling, Empirics, and Policy</t>
+  </si>
+  <si>
+    <t>Willi Semmler</t>
+  </si>
+  <si>
+    <t>Should Charitable and Political Donations Benefit from Similar Tax Treatments? Evidence from a Survey Experiment</t>
+  </si>
+  <si>
+    <t>yuchen huang</t>
+  </si>
+  <si>
+    <t>Returns to wealth for everyone: Long-run evolution of group-specific rates of return along the wealth distribution</t>
+  </si>
+  <si>
+    <t>Filip Novokmet</t>
+  </si>
+  <si>
+    <t>From Housing Gains to Pension Losses: Micro-Macro Integration to Reveal Wealth Inequality Dynamics in Chile</t>
+  </si>
+  <si>
+    <t>Bastián Elías Castro Nofal</t>
+  </si>
+  <si>
+    <t>Drivers of Environmental Consumption Footprint Inequality in Europe</t>
+  </si>
+  <si>
+    <t>Ciccolini Giuseppe</t>
+  </si>
+  <si>
+    <t>How do childhood environments contribute to intergenerational economic mobility? Evidence from 25 years of panel data in Egypt</t>
+  </si>
+  <si>
+    <t>Ragui Assaad</t>
+  </si>
+  <si>
+    <t>The Great Leveler According to HANK</t>
+  </si>
+  <si>
+    <t>Timothy Meyer</t>
+  </si>
+  <si>
+    <t>Political Influence on Agricultural Credit Allocation: Evidence from a Regression Discontinuity Design in India</t>
+  </si>
+  <si>
+    <t>Prosenjit Barman</t>
+  </si>
+  <si>
+    <t>Political Instability, Urban Informality, and Labor Markets: Evidence from Egypt</t>
+  </si>
+  <si>
+    <t>Dima El Hariri</t>
+  </si>
+  <si>
+    <t>Is There Really a Child Penalty in the  Long Run? New Evidence from IVF Treatments</t>
+  </si>
+  <si>
+    <t>Eric Plug</t>
+  </si>
+  <si>
+    <t>Persistent inequalities in exposure to extreme climate events over the 21st century in Europe</t>
+  </si>
+  <si>
+    <t>Mehdi Mikou</t>
+  </si>
+  <si>
+    <t>The rich, the poor and the cleaners A multinational comparison of domestic service and inequality</t>
+  </si>
+  <si>
+    <t>Paul Segal</t>
+  </si>
+  <si>
+    <t>Gateways, Funnels, and Stackers:  How People Hide Property Ownership through Offshore Structures</t>
+  </si>
+  <si>
+    <t>Kristin Surak</t>
+  </si>
+  <si>
+    <t>First to Wake-Up, Last to Eat: Evidence of Disproportionate Morning Penalties on Women in India</t>
+  </si>
+  <si>
+    <t>Udayan Rathore</t>
+  </si>
+  <si>
+    <t>Child Deprivation and Early Educational Outcomes: Evidence from Young Lives, India</t>
+  </si>
+  <si>
+    <t>Ellanki Revathi</t>
+  </si>
+  <si>
+    <t>Geographic inequalities in accessibility of essential services</t>
+  </si>
+  <si>
+    <t>Vanda Almeida</t>
+  </si>
+  <si>
+    <t>Inequality of Opportunity in Labor Markets: A Comparative Analysis of Employment and Wage Disparities in Egypt, Jordan, and Sudan</t>
+  </si>
+  <si>
+    <t>Soufiane Ben Khali</t>
+  </si>
+  <si>
+    <t>A Political Economy Definition of the Middle Class</t>
+  </si>
+  <si>
+    <t>Alejandro Corvalán</t>
+  </si>
+  <si>
+    <t>Did Classical Capitalism Ever Exist? New Evidence from Income Tax and Census Microdata from the USA (1936-1980)</t>
+  </si>
+  <si>
+    <t>Miguel Artola</t>
+  </si>
+  <si>
+    <t>Unequal Regimes, Profitability and its Consequences: Evidence from 129 countries</t>
+  </si>
+  <si>
+    <t>Rishabh Kumar</t>
+  </si>
+  <si>
+    <t>Biased Information, Biased Preferences: How Fragmented Media Environments Undermine Support for Redistribution</t>
+  </si>
+  <si>
+    <t>Oscar Barrera Rodriguez</t>
+  </si>
+  <si>
+    <t>Shaping women's fortunes: inheritance and gender disparities</t>
+  </si>
+  <si>
+    <t>Naomi Crowther</t>
+  </si>
+  <si>
+    <t>The Distribution and Taxation of Inheritances: Microsimulation Evidence for a Common European Inheritance Tax</t>
+  </si>
+  <si>
+    <t>Klaus Grünberger</t>
+  </si>
+  <si>
+    <t>Wealth Inequality, Asset Price Bubbles and Financial Crises</t>
+  </si>
+  <si>
+    <t>Edison Jakurti</t>
+  </si>
+  <si>
+    <t>Rising Gaps, Falling Concentration: Wealth Inequality and Portfolio Diffusion in Sweden</t>
+  </si>
+  <si>
+    <t>Paula Roth</t>
+  </si>
+  <si>
+    <t>Housing Expenses and the Evolution of Income Inequality in Spain</t>
+  </si>
+  <si>
+    <t>Guillermo Lobo</t>
+  </si>
+  <si>
+    <t>The Impact of Extreme Climate Events on Income Distribution in Italy: A Municipality-Level Analysis</t>
+  </si>
+  <si>
+    <t>Matteo Coronese</t>
+  </si>
+  <si>
+    <t>The Wealth Inequality of Real Estate: Other Real Estate and Its Role in Wealth Concentration</t>
+  </si>
+  <si>
+    <t>Pietro Valetto</t>
+  </si>
+  <si>
+    <t>Addressing labour share in Southeast Asia: Malaysian Anomaly and Current Reform</t>
+  </si>
+  <si>
+    <t>Shazrul Suhaimi</t>
+  </si>
+  <si>
+    <t>Turbulence in Taxation: A Study on Tax Avoidance with Private Jets</t>
+  </si>
+  <si>
+    <t>Düzgün Dilsiz</t>
+  </si>
+  <si>
+    <t>Perceptions of Undeserved Inequality Make Europeans More Vulnerable to Populist Narratives</t>
+  </si>
+  <si>
+    <t>Robin Maialeh</t>
+  </si>
+  <si>
+    <t>Assessing the statistical significance of inequality differences: the problem of heavy tails</t>
+  </si>
+  <si>
+    <t>Nicolas Hérault</t>
+  </si>
+  <si>
+    <t>Optimal Transport and the Measurement of Inequality</t>
+  </si>
+  <si>
+    <t>Tommaso Coen</t>
+  </si>
+  <si>
+    <t>Post-growth mitigation scenarios to reduce multidimensional inequalities between world regions</t>
+  </si>
+  <si>
+    <t>Gabriele Dabbaghian</t>
+  </si>
+  <si>
+    <t>Redistribution, Taxes, and Gender Gaps: Evidence from Top Income Adjustments in Chile</t>
+  </si>
+  <si>
+    <t>Rafael Carranza</t>
+  </si>
+  <si>
+    <t>Toward a Theory of the Evolution of the Global Political Economy: Exploring the Effect of ‘Varieties of Capitalism’ on Equality and Sustainability</t>
+  </si>
+  <si>
+    <t>Garry Piepenbrock</t>
+  </si>
+  <si>
+    <t>Equality and Development: A Comparative &amp; Historical Perspective 1800-2025</t>
+  </si>
+  <si>
+    <t>Manuel Esteban Arias-Osorio</t>
+  </si>
+  <si>
+    <t>From Polarization to Dualization : How Stratification Filters Automation Shocks in Korea</t>
+  </si>
+  <si>
+    <t>Hoyeon Lee</t>
+  </si>
+  <si>
+    <t>Domestic Inequality and Global Imbalances</t>
+  </si>
+  <si>
+    <t>Jan Mazza</t>
+  </si>
+  <si>
+    <t>The Democratic Welfare State: How does the Welfare State moderate Political Participation Gaps between Labor Market Insiders and Outsiders?</t>
+  </si>
+  <si>
+    <t>Nastia Nedjai</t>
+  </si>
+  <si>
+    <t>Measuring Inflation Inequality in India: A State-level Analysis</t>
+  </si>
+  <si>
+    <t>Prachi Bansal</t>
+  </si>
+  <si>
+    <t>Inequality measurement for count data: theory and application to inequality in household sizes across the world</t>
+  </si>
+  <si>
+    <t>Gaston Yalonetzky</t>
+  </si>
+  <si>
+    <t>Female Angel Investors Challenge the Gender Roles: An Analysis of Gender Dynamics Between Investors and Founders</t>
+  </si>
+  <si>
+    <t>Yunus Isik</t>
+  </si>
+  <si>
+    <t>Global South dependence on production in the core: an empirical assessment of trends from 1995-2020</t>
+  </si>
+  <si>
+    <t>Omer Tayyab</t>
+  </si>
+  <si>
+    <t>Who Owns Cryptocurrency?</t>
+  </si>
+  <si>
+    <t>Andreas Økland</t>
+  </si>
+  <si>
+    <t>Are US Billionaires' Unrealized Capital Gains "Paper Gains"?</t>
+  </si>
+  <si>
+    <t>Jasper Boll</t>
+  </si>
+  <si>
+    <t>Land for Opportunity? Deprivation and Immobility in Rural India</t>
+  </si>
+  <si>
+    <t>Vibhu Pratyush</t>
+  </si>
+  <si>
+    <t>The Network Origins of Carbon Pricing Regressivity</t>
+  </si>
+  <si>
+    <t>Bernardo Fernandes</t>
+  </si>
+  <si>
+    <t>Housing Inheritances and the Spatial Misallocation of Talent: A Geography of Missed Opportunities</t>
+  </si>
+  <si>
+    <t>Bluebery Planterose</t>
+  </si>
+  <si>
+    <t>Does Educational Mismatch Penalize Women Less? Evidence from India’s Labour Market</t>
+  </si>
+  <si>
+    <t>Soumyaranjan Mukherjee</t>
+  </si>
+  <si>
+    <t>Closing the gender time gap: how formal childcare affects parental work and care dynamics</t>
+  </si>
+  <si>
+    <t>Sophie Achleitner</t>
+  </si>
+  <si>
+    <t>Societal Explanations of Economic Inequality</t>
+  </si>
+  <si>
+    <t>Magdalena Wasilewska</t>
+  </si>
+  <si>
+    <t>Housing Returns across the Income Distribution</t>
+  </si>
+  <si>
+    <t>Natalia Khorunzhina</t>
+  </si>
+  <si>
+    <t>Multidimensional Inequality in Latin America</t>
+  </si>
+  <si>
+    <t>Andres Espejo</t>
+  </si>
+  <si>
+    <t>Six Decades of Unequal Growth: Income and Wealth Inequality in Turkey, 1968–2022</t>
+  </si>
+  <si>
+    <t>Enes Isik</t>
+  </si>
+  <si>
+    <t>Ideological Shifts and Wealth Dynamics: Unraveling the Century-Long Accumulation of Chinese National Wealth, 1911-2020</t>
+  </si>
+  <si>
+    <t>Zhexun Mo</t>
+  </si>
+  <si>
+    <t>Intergenerational Wealth Mobility over Two Centuries: Evolution and Determinants</t>
+  </si>
+  <si>
+    <t>Jonathan Goupille-Lebret</t>
+  </si>
+  <si>
+    <t>Online media and polarization: Theory and cross-country evidence</t>
+  </si>
+  <si>
+    <t>Jun HU</t>
+  </si>
+  <si>
+    <t>The Deepening Divide Within the Rich as a Key Driver of U.S. Economic Inequality</t>
+  </si>
+  <si>
+    <t>Hyeongwoo Kim</t>
+  </si>
+  <si>
+    <t>Should capital gains be tax privileged?</t>
+  </si>
+  <si>
+    <t>Andrew Lonsdale</t>
+  </si>
+  <si>
+    <t>Towards Narratives of Inequality</t>
+  </si>
+  <si>
+    <t>Frank Cowell - Emmanuel Flachaire</t>
+  </si>
+  <si>
+    <t>Inequality in BTT Bargaining? Allocation of Taxing Rights between Developed and Developing Countries</t>
+  </si>
+  <si>
+    <t>Celine Azemar</t>
+  </si>
+  <si>
+    <t>Residual Income Progression in the Twentieth and Twenty-First Centuries</t>
+  </si>
+  <si>
+    <t>Marcelo Montes Muñoz</t>
+  </si>
+  <si>
+    <t>Impact of financial support for entrepreneurship on economic performance  in Senegal: The case of PAVIE</t>
+  </si>
+  <si>
+    <t>Boina Yasser</t>
+  </si>
+  <si>
+    <t>Does the apple fall far from the tree? New evidence on intergenerational social mobility across OECD countries</t>
+  </si>
+  <si>
+    <t>Tomomi Tanaka</t>
+  </si>
+  <si>
+    <t>The Extraordinary Rise in the Wealth of Older American Households</t>
+  </si>
+  <si>
+    <t>Edward Wolff</t>
+  </si>
+  <si>
+    <t>Gender Norms, Social Pressure, and the Gender Gap in Turnout: Evidence from Swiss Elections</t>
+  </si>
+  <si>
+    <t>Alda Marchese</t>
+  </si>
+  <si>
+    <t>Inequality and Insurgency</t>
+  </si>
+  <si>
+    <t>Etienne Le Rossignol</t>
+  </si>
+  <si>
+    <t>Do Institutions Remove Inflation’s Grease? Evidence from Brazil’s Indexed Minimum Wage</t>
+  </si>
+  <si>
+    <t>Isabel Di Tella</t>
+  </si>
+  <si>
+    <t>Wealth Inequality and Welfare States: Pension systems, the Public-Private Mix, and Augmented Wealth in Old Age</t>
+  </si>
+  <si>
+    <t>Kun Lee</t>
+  </si>
+  <si>
+    <t>Born Here, Raised There: Regional Mobility And Intergenerational Transmission of Education in Europe</t>
+  </si>
+  <si>
+    <t>Enkelejda Havari</t>
+  </si>
+  <si>
+    <t>Spatial income inequality in Germany, 1957-2021</t>
+  </si>
+  <si>
+    <t>Thomas Rieger</t>
+  </si>
+  <si>
+    <t>From Lion Rock to Locked Gates: The Decline of Upward Mobility in Hong Kong</t>
+  </si>
+  <si>
+    <t>Zhejin Zhao</t>
+  </si>
+  <si>
+    <t>Extreme Weather And Economic Insecurity in Malawi: The Impact of Cyclone Ana</t>
+  </si>
+  <si>
+    <t>Raffaela Grigolli Cesar</t>
+  </si>
+  <si>
+    <t>Public Acceptance of International Redistribution in High-Income Countries</t>
+  </si>
+  <si>
+    <t>Adrien Fabre</t>
+  </si>
+  <si>
+    <t>Wealth Inequality in England 1258-1858: Evidence from Wills</t>
+  </si>
+  <si>
+    <t>Neil Cummins</t>
+  </si>
+  <si>
+    <t>Divide in the fields: A study of global agricultural land inequality</t>
+  </si>
+  <si>
+    <t>Marcus Alberic O'Neill</t>
+  </si>
+  <si>
+    <t>The Good Council: Deliberating Inequality in a Field Experiment</t>
+  </si>
+  <si>
+    <t>Severin Rapp</t>
+  </si>
+  <si>
+    <t>Keynes's Vision of Inequality (And Why it Matters)</t>
+  </si>
+  <si>
+    <t>Marc Morgan</t>
+  </si>
+  <si>
+    <t>Status Inequality and Ideology: How Social Hierarchy shaped Redistribution in India</t>
+  </si>
+  <si>
+    <t>Poulomi Chakrabarti</t>
+  </si>
+  <si>
+    <t>Do Poverty Alleviation Policies Enhance Household Resilience to Poverty? Evidence from Bangladesh</t>
+  </si>
+  <si>
+    <t>Salauddin Tauseef</t>
+  </si>
+  <si>
+    <t>Changing Minds: How Academic Fields Shape Political Attitudes</t>
+  </si>
+  <si>
+    <t>Yoav Goldstein</t>
+  </si>
+  <si>
+    <t>Wealthier and Healthier? Place-Based Mechanisms in the  Wealth-Health Relationship</t>
+  </si>
+  <si>
+    <t>Sehyun Hong</t>
+  </si>
+  <si>
+    <t>Income Inequality Early in Life: Underage Children as Owners of Privately Held Firms</t>
+  </si>
+  <si>
+    <t>Terhi Ravaska</t>
+  </si>
+  <si>
+    <t>Does Financial Inclusion Mitigate Social Exclusion?</t>
+  </si>
+  <si>
+    <t>Rikhia Bhukta</t>
+  </si>
+  <si>
+    <t>Playing the birth lottery in Europe</t>
+  </si>
+  <si>
+    <t>Annaelena Valentini</t>
+  </si>
+  <si>
+    <t>Corruption Information and Inequality Perceptions: Causal Evidence from Central and Eastern European Democracies</t>
+  </si>
+  <si>
+    <t>Denis Ivanov</t>
+  </si>
+  <si>
+    <t>A Golden Age for All?  Income Inequality and Social Classes in Italy, 1951-1973</t>
+  </si>
+  <si>
+    <t>Giacomo Gabbuti</t>
+  </si>
+  <si>
+    <t>Demographic Change and Intergenerational Transmission.  With an application to China</t>
+  </si>
+  <si>
+    <t>Dirk Van de Gaer</t>
+  </si>
+  <si>
+    <t>Measuring Political Inequality: Roads Distribution and Developement Aid Effectiveness in Indonesia</t>
+  </si>
+  <si>
+    <t>Nathan Peng Li</t>
+  </si>
+  <si>
+    <t>How do Development Assistance and Illicit Financial Flows Affect Income Distributions?</t>
+  </si>
+  <si>
+    <t>Magdalene Silberberger</t>
+  </si>
+  <si>
+    <t>Cutting hours through outsourcing</t>
+  </si>
+  <si>
+    <t>Ulysse Lojkine</t>
+  </si>
+  <si>
+    <t>Multidimensional Inequality among the Elderly in the United States</t>
+  </si>
+  <si>
+    <t>Shatakshee Dhongde</t>
+  </si>
+  <si>
+    <t>Income distribution in Poland, 1924–1945: pro-poor growth, ethnic inequality, and the consequences of World War II and the Holocaust</t>
+  </si>
+  <si>
+    <t>Marcin Wroński</t>
+  </si>
+  <si>
+    <t>From Roots to Returns: Does Migration Improve Economic Welfare? Evidence from India</t>
+  </si>
+  <si>
+    <t>Saakshi Duseja</t>
+  </si>
+  <si>
+    <t>Better Call Bill? Philanthropy and Preferences for  Taxing the Super-rich.</t>
+  </si>
+  <si>
+    <t>César Fuster Llamazares</t>
+  </si>
+  <si>
+    <t>Personal Distribution of Income and Wealth of the Brazilian Population</t>
+  </si>
+  <si>
+    <t>Rafael de Acypreste Monteiro Rocha</t>
+  </si>
+  <si>
+    <t>The Climate Cost of Inequality: Trade-offs and Structural Effects</t>
+  </si>
+  <si>
+    <t>Svenja Fletchner</t>
+  </si>
+  <si>
+    <t>Robust Estimation of Private Business Wealth</t>
+  </si>
+  <si>
+    <t>Simon Toussaint</t>
+  </si>
+  <si>
+    <t>Top Incomes in Twentieth-Century Mexico: New Evidence from Tax Records</t>
+  </si>
+  <si>
+    <t>Enrique de la Rosa-Ramos</t>
+  </si>
+  <si>
+    <t>The Global Distribution of Human and Nonhuman Wealth</t>
+  </si>
+  <si>
+    <t>Olle Hammar</t>
+  </si>
+  <si>
+    <t>Recent Trends in Income Concentration in Japan, 2008-2023:  New Estimates of Top Fiscal Income Shares and Top National Income Shares</t>
+  </si>
+  <si>
+    <t>Chiaki Moriguchi</t>
+  </si>
+  <si>
+    <t>Automation and Inequality Within Firms: Evidence from South Africa</t>
+  </si>
+  <si>
+    <t>Rafael Consentino de la Vega</t>
+  </si>
+  <si>
+    <t>Global Mobility Ginis: The Inequality of International Mobility between 186 Countries (1995-2022)</t>
+  </si>
+  <si>
+    <t>Ettore Recchi</t>
+  </si>
+  <si>
+    <t>From Flat to Fair? The Effects of a Progressive Tax Reform</t>
+  </si>
+  <si>
+    <t>Guillermo Cruces</t>
+  </si>
+  <si>
+    <t>From Aristocratic Estates to Bureaucratic Fortunes: Intergenerational Wealth in Georgia (1900–2020)</t>
+  </si>
+  <si>
+    <t>Alexander Tsagareli</t>
+  </si>
+  <si>
+    <t>Inheritance Tax Around the Globe Over Two Centuries: Revenue and Distributional Implications</t>
+  </si>
+  <si>
+    <t>Luca Giangregorio</t>
+  </si>
+  <si>
+    <t>Housing costs and the distribution of income.</t>
+  </si>
+  <si>
+    <t>Pedro Salas Rojo</t>
+  </si>
+  <si>
+    <t>Limits to VAT Self-Enforcement: Role of Network Frictions in Compliance</t>
+  </si>
+  <si>
+    <t>Bhanu Gupta</t>
+  </si>
+  <si>
+    <t>Land Inequality in India</t>
+  </si>
+  <si>
+    <t>Nitin Kumar Bharti</t>
+  </si>
+  <si>
+    <t>Return on team moves</t>
+  </si>
+  <si>
+    <t>Olivier Godechot</t>
+  </si>
+  <si>
+    <t>Majority in 40 Countries Support Unprecedented Coordinated Billionaire Tax Discussed by G20</t>
+  </si>
+  <si>
+    <t>Morten Nyborg Støstad</t>
+  </si>
+  <si>
+    <t>Mind the gap and the map: Measuring distributional and spatial income polarization</t>
+  </si>
+  <si>
+    <t>Sergio Rey</t>
+  </si>
+  <si>
+    <t>Long-term Land Inequality and Post-Colonial Land Reform in Egypt (1896-2020)</t>
+  </si>
+  <si>
+    <t>Rowaida Moshrif</t>
+  </si>
+  <si>
+    <t>Profit Shifting via Carbon Emission Trading: First Indications</t>
+  </si>
+  <si>
+    <t>Alison Schultz</t>
+  </si>
+  <si>
+    <t>Welfare Policy, Education and Inclusive Growth: Evidence from India</t>
+  </si>
+  <si>
+    <t>Amartya Paul</t>
+  </si>
+  <si>
+    <t>Ready to switch? Fairness implications from heterogeneous access to climate-friendly substitutes</t>
+  </si>
+  <si>
+    <t>Franziska Funke</t>
+  </si>
+  <si>
+    <t>The Shared Socio-economic Pathways of global welfare: A sub-national database integrating income inequality and  climate change impacts</t>
+  </si>
+  <si>
+    <t>Fabrice Murtin</t>
+  </si>
+  <si>
+    <t>Enforcing Taxes on Cryptocurrencies</t>
+  </si>
+  <si>
+    <t>Mona Barake</t>
+  </si>
+  <si>
+    <t>Job Composition, Gender and Income Inequality in the Long Run: Sweden, 1870–1950</t>
+  </si>
+  <si>
+    <t>Jakob Molinder</t>
+  </si>
+  <si>
+    <t>Does Discrimination Exist in the Market for Educational loans? Experimental Evidence from India’s Caste System</t>
+  </si>
+  <si>
+    <t>Navjot Sangwan</t>
+  </si>
+  <si>
+    <t>Tax Incentives or Political Motivations? Evidence from Corporate Contributions</t>
+  </si>
+  <si>
+    <t>Malka Guillot</t>
+  </si>
+  <si>
+    <t>Life-time Income Inequality in Denmark</t>
+  </si>
+  <si>
+    <t>Jonas Maibom</t>
+  </si>
+  <si>
+    <t>Taxing the Rich in Latin America: Effects of a Wealth Tax on Revenue and Distribution</t>
+  </si>
+  <si>
+    <t>Mauricio De Rosa</t>
+  </si>
+  <si>
+    <t>Economic Inequality and Biodiversity Loss. An empirical analysis of Keo Seima Wildlife Sanctuary, 2012-2022</t>
+  </si>
+  <si>
+    <t>Paulo Santos</t>
+  </si>
+  <si>
+    <t>Luxury for All: A Theory of Public Provision and Inequality</t>
+  </si>
+  <si>
+    <t>Yann Perdereau</t>
+  </si>
+  <si>
+    <t>Racial Inequality in France</t>
+  </si>
+  <si>
+    <t>Yajna Govind</t>
+  </si>
+  <si>
+    <t>Work-From-Home and Intergenerational Mobility</t>
+  </si>
+  <si>
+    <t>Francesco Saverio Lenzi</t>
+  </si>
+  <si>
+    <t>Spatial wage inequality in North America and Western Europe: changes between and within local labour markets 1975-2019</t>
+  </si>
+  <si>
+    <t>Pawel Bukowski</t>
+  </si>
+  <si>
+    <t>Redressing hyper-globalisation and the inequities systemically generated in GVCs: Multilateral efforts at the UN</t>
+  </si>
+  <si>
+    <t>Gabriele Koehler</t>
+  </si>
+  <si>
+    <t>Credit Redistribution in the Age of Fintech:  Climate Shocks and Inequality in Rural India</t>
+  </si>
+  <si>
+    <t>Anand Mathew</t>
+  </si>
+  <si>
+    <t>Unfulfilled Prophecy: The Moderating Role of Meritocratic Beliefs in the Relationship Between Inequality and Subjective Well-Being</t>
+  </si>
+  <si>
+    <t>Camila Bidó</t>
+  </si>
+  <si>
+    <t>Global Working Hours</t>
+  </si>
+  <si>
+    <t>Amory Gethin</t>
+  </si>
+  <si>
+    <t>Preferences for redistribution policies among politicians and citizens</t>
+  </si>
+  <si>
+    <t>Javier Olivera</t>
+  </si>
+  <si>
+    <t>Guns and Gains: Human Capital Effects of Exposure to Counterinsurgency Operations</t>
+  </si>
+  <si>
+    <t>Punarjit Roychowdhury</t>
+  </si>
+  <si>
+    <t>Backlash or Bonding? Effect of Integration Policies in a Context of Affirmative Action</t>
+  </si>
+  <si>
+    <t>Balasai Vanukuri</t>
+  </si>
+  <si>
+    <t>Dissecting the gender gap in intergenerational transfers: the case of Germany</t>
+  </si>
+  <si>
+    <t>Eva Sierminska</t>
+  </si>
+  <si>
+    <t>The Fundamental Law of Oligarchy: on the Transnational Constitutional Foundations of the Inequality Crisis</t>
+  </si>
+  <si>
+    <t>Timothy K. Kuhner</t>
+  </si>
+  <si>
+    <t>Poverty, Inequality, and Working Hours: Evidence on Veblen Effects from Labour Markets in India</t>
+  </si>
+  <si>
+    <t>Karthikeya Naraparaju</t>
+  </si>
+  <si>
+    <t>Sectoral Bargaining and the Wage Structure</t>
+  </si>
+  <si>
+    <t>Alexander Busch</t>
+  </si>
+  <si>
+    <t>Ancestral Inequality and Preferences for Redistribution</t>
+  </si>
+  <si>
+    <t>Graziella Bertocchi</t>
+  </si>
+  <si>
+    <t>Caste Reparations: Economic Advancement, Social Concord, and Policy Backlash</t>
+  </si>
+  <si>
+    <t>Gautam Nair</t>
+  </si>
+  <si>
+    <t>Does inequalities in access smartphone and internet lead to poor learning outcomes? Evidence from rural India</t>
+  </si>
+  <si>
+    <t>Pradeep Kumar Choudhury</t>
+  </si>
+  <si>
+    <t>Unifying Absolute and Relative Poverty Measurement: A Strict Separation Approach</t>
+  </si>
+  <si>
+    <t>Michail Moatsos</t>
+  </si>
+  <si>
+    <t>Inequality and Redistribution in the Netherlands</t>
+  </si>
+  <si>
+    <t>Wouter Leenders</t>
+  </si>
+  <si>
+    <t>Attribution Bias by Gender</t>
+  </si>
+  <si>
+    <t>Karmini Sharma</t>
+  </si>
+  <si>
+    <t>Belgian wealth inequality, 1935-2022</t>
+  </si>
+  <si>
+    <t>Arthur Apostel</t>
+  </si>
+  <si>
+    <t>Transitions toward Dematerialization and Environmental Inequalities in Latin America: CO₂ Emissions, Material Consumption and Material Footprint in the Framework of the World Inequality Conference 2026 (1970–2024)</t>
+  </si>
+  <si>
+    <t>Fander Falconi Benitez</t>
+  </si>
+  <si>
+    <t>Go Your Own Way? Peer Effects, School Choice, and Educational Inequality</t>
+  </si>
+  <si>
+    <t>Inbar Amit</t>
+  </si>
+  <si>
+    <t>Estimating the Muslim Wage Penalty</t>
+  </si>
+  <si>
+    <t>Pauline Corblet</t>
+  </si>
+  <si>
+    <t>Has oil richness been a force for income equality in Venezuela over the long term?</t>
+  </si>
+  <si>
+    <t>Pablo Astorga</t>
+  </si>
+  <si>
+    <t>Offshoring wage inequality in tax havens</t>
+  </si>
+  <si>
+    <t>Gabriel Smagghue</t>
+  </si>
+  <si>
+    <t>Who benefits from payroll tax subsidies for older workers? Incidence at the individual and firm level</t>
+  </si>
+  <si>
+    <t>Alba Vazquez Garcia</t>
+  </si>
+  <si>
+    <t>Perceived Intergenerational Mobility in Latin America</t>
+  </si>
+  <si>
+    <t>Valentina Gabrielli</t>
+  </si>
+  <si>
+    <t>Income Shocks, Economic Inequality, and Political Realignment: Voter Turnout and the Shift to a Multi-Party System in Costa Rica</t>
+  </si>
+  <si>
+    <t>Alvaro Zuniga-Cordero</t>
+  </si>
+  <si>
+    <t>Understanding distortions in Gini coefficient comparisons:   Isogini measures of income and wealth distributions with WID 2010-2020</t>
+  </si>
+  <si>
+    <t>Louis Chauvel</t>
+  </si>
+  <si>
+    <t>Income Inequality in a Nordic Welfare State: Finnish Distributional National Accounts</t>
+  </si>
+  <si>
+    <t>Toni Juuti</t>
+  </si>
+  <si>
+    <t>Cultural Constraints on Women’s Productivity: Evidence from World Bank Lending</t>
+  </si>
+  <si>
+    <t>Michele Valsecchi</t>
+  </si>
+  <si>
+    <t>The impact of freshwater changes on economic production worldwide</t>
+  </si>
+  <si>
+    <t>Anna Reckwitz</t>
+  </si>
+  <si>
+    <t>Who Benefits from Affirmative Action? Sub-Caste Inequality in India</t>
+  </si>
+  <si>
+    <t>Pawandeep Kaur</t>
+  </si>
+  <si>
+    <t>Circumstance Elasticity of Income</t>
+  </si>
+  <si>
+    <t>Gaurav Datt</t>
+  </si>
+  <si>
+    <t>Saving Rate Heterogeneity across the Wealth (Rank) Distribution in the United States</t>
+  </si>
+  <si>
+    <t>‘Diminishing One Gap, Widening Another’: Unintended Consequences of Adult Literacy on Medium-Term Child Dropouts in India</t>
+  </si>
+  <si>
+    <t>Sulagna Bhattacharya</t>
+  </si>
+  <si>
+    <t>Health In-Kind Benefits are Pro-Poor: Measuring their Distributional Impact in the EU</t>
+  </si>
+  <si>
+    <t>Gemma Riera Mallol</t>
+  </si>
+  <si>
+    <t>Earning disparities between migrant and non-migrant workers: A quantile decomposition analysis of the Indian Labour Market</t>
+  </si>
+  <si>
+    <t>Vijay Kumar</t>
+  </si>
+  <si>
+    <t>Model Uncertainty and Measures of Inequality of Opportunity</t>
+  </si>
+  <si>
+    <t>Andros Kourtellos</t>
+  </si>
+  <si>
+    <t>The Anti-Austerity Party: A Neglected Party of the Working Class</t>
+  </si>
+  <si>
+    <t>Panos Tsoukalis</t>
+  </si>
+  <si>
+    <t>Why Awareness Needs Inclusion: Evidence from a Menstrual Health Campaigns in Nepal</t>
+  </si>
+  <si>
+    <t>Silvia Castro</t>
+  </si>
+  <si>
+    <t>The Kuznets Curve with No Return: The Industrial Revolution and Wealth Inequality</t>
+  </si>
+  <si>
+    <t>Timo Stieglitz</t>
+  </si>
+  <si>
+    <t>Households' food carbon footprints</t>
+  </si>
+  <si>
+    <t>Ondine Berland</t>
+  </si>
+  <si>
+    <t>Wealth Inequality Trends Around the World: a first view from the GC Wealth Project data</t>
+  </si>
+  <si>
+    <t>Franziska Disslbacher</t>
+  </si>
+  <si>
+    <t>Exposure to Inequality, Human Capital Investment, and Labor Market Outcomes</t>
+  </si>
+  <si>
+    <t>Petter Lundborg</t>
+  </si>
+  <si>
+    <t>Distribution of household wealth in line with national accounts: Methodology and results from the 2025 experimental data collection</t>
+  </si>
+  <si>
+    <t>Philip Chan</t>
+  </si>
+  <si>
+    <t>Britain's 1986 Big Bang: how state-led financial deregulation durably boosted inequality and hampered long-term economic welfare in the UK</t>
+  </si>
+  <si>
+    <t>Louis Flamencourt</t>
+  </si>
+  <si>
+    <t>Tax Progressivity and Inequality in Brazil: Evidence from Integrated Administrative Data</t>
+  </si>
+  <si>
+    <t>Theo Palomo</t>
+  </si>
+  <si>
+    <t>Mapping subnational price differences across countries: Evidence from OECD regions</t>
+  </si>
+  <si>
+    <t>Juergen Amann</t>
+  </si>
+  <si>
+    <t>Global Evidence on Gender Gaps and Child Poverty in Consumption</t>
+  </si>
+  <si>
+    <t>Maira Colacce</t>
+  </si>
+  <si>
+    <t>Regional wealth inequality in Spain: Evidence from the Spain wealth Atlas</t>
+  </si>
+  <si>
+    <t>Dmitry Petrov</t>
+  </si>
+  <si>
+    <t>Carbon Inequality in the EU</t>
+  </si>
+  <si>
+    <t>Berr Nicole</t>
+  </si>
+  <si>
+    <t>Climate Change, Labour Markets, and Wage Inequality</t>
+  </si>
+  <si>
+    <t>Romano Tarsia</t>
+  </si>
+  <si>
+    <t>Who Owns the Green Transition? Unequal Access to Finance in a Dynamic Framework</t>
+  </si>
+  <si>
+    <t>Morgane Gonon</t>
+  </si>
+  <si>
+    <t>How Much Can Elites Extract? Subsistence Constraints and the Long-Run Evolution of Top Incomes, 1700-2022</t>
+  </si>
+  <si>
+    <t>Andres Irarrazaval Garcia Huidobro</t>
+  </si>
+  <si>
+    <t>Local Inequality and the Backlash Against Global Economic Governance</t>
+  </si>
+  <si>
+    <t>alexander wais</t>
+  </si>
+  <si>
+    <t>The Geography of Fuel Tax Incidence</t>
+  </si>
+  <si>
+    <t>Giulia Tani</t>
+  </si>
+  <si>
+    <t>Structural Transformation and Top Income Inequality</t>
+  </si>
+  <si>
+    <t>Martin Shu</t>
+  </si>
+  <si>
+    <t>From Creative Destruction to Creative Appropriation – Rethinking Growth in Intellectual Monopoly Capitalism</t>
+  </si>
+  <si>
+    <t>Linus Zechlin</t>
+  </si>
+  <si>
+    <t>Income shocks and gender gaps: long-run evidence from India</t>
+  </si>
+  <si>
+    <t>Angelica Bozzi</t>
+  </si>
+  <si>
+    <t>Drivers of Lifetime Earnings and Wealth: Skills, Frictions and Choices</t>
+  </si>
+  <si>
+    <t>Francesco Del Prato</t>
+  </si>
+  <si>
+    <t>When Trade Compresses: The Impact of Liberalization on Wage Inequality</t>
+  </si>
+  <si>
+    <t>Victor Hernandez Martinez</t>
+  </si>
+  <si>
+    <t>Intergenerational Income Mobility around the World: A Meta-Analysis</t>
+  </si>
+  <si>
+    <t>Louis Sirugue</t>
+  </si>
+  <si>
+    <t>Atlas of the Offshore World</t>
+  </si>
+  <si>
+    <t>Annette Alstadsæter</t>
+  </si>
+  <si>
+    <t>Global estimates of opportunity and mobility: a database</t>
+  </si>
+  <si>
+    <t>Paolo Brunori</t>
+  </si>
+  <si>
+    <t>Prosperity Within Limits? Planetary Habitability, Global Convergence and Structural Transformation, 2026-2100</t>
+  </si>
+  <si>
+    <t>Moritz Odersky</t>
+  </si>
+  <si>
+    <t>The Global Justice Platform: Distributional Pathways, the Global Justice Fund and the New Democratic International Order, 2026-2100</t>
+  </si>
+  <si>
+    <t>Jonas Dietrich</t>
+  </si>
+  <si>
+    <t>Global Labour Hours in Paid and Unpaid Work: Productivity and Structural Transformation, 1800-2100</t>
+  </si>
+  <si>
+    <t>Romaine Loubes</t>
+  </si>
+  <si>
+    <t>Human Capital, Unequal Opportunities and Productivity Convergence: A Global Historical Perspective, 1800-2100</t>
+  </si>
+  <si>
+    <t>Thanasak Mark Jenmana</t>
+  </si>
+  <si>
+    <t>Introduction to AIR: Concept, Approach, and Research Questions</t>
+  </si>
+  <si>
+    <t>Murray Leibbrandt</t>
+  </si>
+  <si>
+    <t>The Latin American (LACIR) example: “here is one we made earlier…”</t>
+  </si>
+  <si>
+    <t>Francisco Ferreira</t>
+  </si>
+  <si>
+    <t>Fairer but Falling Behind: Africa's Inequality Paradox in a Shifting Global Order  -- Rodrigo Oliveira</t>
+  </si>
+  <si>
+    <t>Rodrigo Oliveira</t>
+  </si>
+  <si>
+    <t>Argue, Pledge and Implement: Investigating the Role of Fairness in International Climate Policy</t>
+  </si>
+  <si>
+    <t>Martino Kuntze</t>
+  </si>
+  <si>
+    <t>Quid pro quo? Electoral Donations and Tax Amnesty Programs in Brazil</t>
+  </si>
+  <si>
+    <t>Natalia Ferreira De Carvalho Rodrigues</t>
+  </si>
+  <si>
+    <t>Asset Tests and Household Dissaving: Evidence from Spanish Minimum Income Scheme; Regional wealth inequality in Spain: evidence from the Spain Wealth Atlas</t>
+  </si>
+  <si>
+    <t>Unequal Exchange and North-South Relations: Evidence from Global Trade Flows and the World Balance of Payments 1800-2025</t>
+  </si>
+  <si>
+    <t>Gaston Nievas</t>
+  </si>
+  <si>
+    <t>Capital- and finance-based environmental accounting framework</t>
+  </si>
+  <si>
+    <t>Manuel Tomás</t>
+  </si>
+  <si>
+    <t>When Organized Crime Moves In: Economic and Human Capital Disruption</t>
+  </si>
+  <si>
+    <t>Erika Povea</t>
+  </si>
+  <si>
+    <t>End of Apartheid, Not of Inequality: The Slow Transition in a Segregated Economy</t>
+  </si>
+  <si>
+    <t>Kristina Manysheva</t>
+  </si>
+  <si>
     <t>IssueType</t>
   </si>
   <si>
@@ -21264,112 +22891,10 @@
     <t>Overflow</t>
   </si>
   <si>
-    <t>Rafael Carranza</t>
-  </si>
-  <si>
-    <t>Redistribution, Taxes, and Gender Gaps: Evidence from Top Income Adjustments in Chile</t>
-  </si>
-  <si>
     <t>Session currently exceeds capacity (4); organizer decision required.</t>
   </si>
   <si>
-    <t>Giulia Tani</t>
-  </si>
-  <si>
-    <t>The Geography of Fuel Tax Incidence</t>
-  </si>
-  <si>
-    <t>Garry Piepenbrock</t>
-  </si>
-  <si>
-    <t>Toward a Theory of the Evolution of the Global Political Economy: Exploring the Effect of ‘Varieties of Capitalism’ on Equality and Sustainability</t>
-  </si>
-  <si>
     <t>Session currently exceeds capacity (5); organizer decision required.</t>
-  </si>
-  <si>
-    <t>Annette Alstadsæter</t>
-  </si>
-  <si>
-    <t>Atlas of the Offshore World</t>
-  </si>
-  <si>
-    <t>Julian Koller</t>
-  </si>
-  <si>
-    <t>Inequality and Redistribution in Switzerland: Evidence from Distributional National Accounts</t>
-  </si>
-  <si>
-    <t>Paula Roth</t>
-  </si>
-  <si>
-    <t>Rising Gaps, Falling Concentration: Wealth Inequality and Portfolio Diffusion in Sweden</t>
-  </si>
-  <si>
-    <t>Ararat Gocmen - Clara Martinez-Toledano</t>
-  </si>
-  <si>
-    <t>Private Capital Markets and Inequality</t>
-  </si>
-  <si>
-    <t>Martin Shu</t>
-  </si>
-  <si>
-    <t>Structural Transformation and Top Income Inequality</t>
-  </si>
-  <si>
-    <t>Matteo Coronese</t>
-  </si>
-  <si>
-    <t>The Impact of Extreme Climate Events on Income Distribution in Italy: A Municipality-Level Analysis</t>
-  </si>
-  <si>
-    <t>Raffaela Grigolli Cesar</t>
-  </si>
-  <si>
-    <t>Extreme Weather And Economic Insecurity in Malawi: The Impact of Cyclone Ana</t>
-  </si>
-  <si>
-    <t>Udayan Rathore</t>
-  </si>
-  <si>
-    <t>First to Wake-Up, Last to Eat: Evidence of Disproportionate Morning Penalties on Women in India</t>
-  </si>
-  <si>
-    <t>Samuel Kofi Tetteh-Baah</t>
-  </si>
-  <si>
-    <t>Measuring Global Inequality: How accounting for inequality within the household affects the global profile</t>
-  </si>
-  <si>
-    <t>Magdalene Silberberger</t>
-  </si>
-  <si>
-    <t>How do Development Assistance and Illicit Financial Flows Affect Income Distributions?</t>
-  </si>
-  <si>
-    <t>Dongwoong Seo</t>
-  </si>
-  <si>
-    <t>Understanding Survey Income Errors Using Linked Administrative Data</t>
-  </si>
-  <si>
-    <t>Pauline Corblet</t>
-  </si>
-  <si>
-    <t>Estimating the Muslim Wage Penalty</t>
-  </si>
-  <si>
-    <t>Michail Moatsos</t>
-  </si>
-  <si>
-    <t>Unifying Absolute and Relative Poverty Measurement: A Strict Separation Approach</t>
-  </si>
-  <si>
-    <t>Laura Pereira</t>
-  </si>
-  <si>
-    <t>Solving science conundrums in the climate-nature-equity polycrisis: The need for transformative, socially just, climate and biodiversity scenarios</t>
   </si>
   <si>
     <t>SlotCollision</t>
@@ -30546,6 +32071,2196 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B272"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="72.7109375" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="8" t="s">
+        <v>783</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="8" t="s">
+        <v>785</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="8" t="s">
+        <v>787</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="8" t="s">
+        <v>789</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="8" t="s">
+        <v>791</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="8" t="s">
+        <v>793</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="8" t="s">
+        <v>795</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="8" t="s">
+        <v>797</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="8" t="s">
+        <v>799</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="8" t="s">
+        <v>801</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="8" t="s">
+        <v>803</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="8" t="s">
+        <v>805</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="8" t="s">
+        <v>807</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="8" t="s">
+        <v>809</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="8" t="s">
+        <v>811</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="8" t="s">
+        <v>813</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="8" t="s">
+        <v>815</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="8" t="s">
+        <v>817</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="8" t="s">
+        <v>819</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="8" t="s">
+        <v>821</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="8" t="s">
+        <v>823</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="8" t="s">
+        <v>825</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="8" t="s">
+        <v>829</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="8" t="s">
+        <v>831</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="8" t="s">
+        <v>833</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="8" t="s">
+        <v>835</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="8" t="s">
+        <v>837</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="8" t="s">
+        <v>839</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="8" t="s">
+        <v>841</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="8" t="s">
+        <v>843</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="8" t="s">
+        <v>845</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="8" t="s">
+        <v>847</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="8" t="s">
+        <v>849</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="8" t="s">
+        <v>851</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="8" t="s">
+        <v>853</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="8" t="s">
+        <v>855</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="8" t="s">
+        <v>857</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="8" t="s">
+        <v>859</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="8" t="s">
+        <v>861</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="8" t="s">
+        <v>863</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="8" t="s">
+        <v>865</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="8" t="s">
+        <v>867</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="8" t="s">
+        <v>869</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="8" t="s">
+        <v>871</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="8" t="s">
+        <v>873</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="8" t="s">
+        <v>875</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="8" t="s">
+        <v>877</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="8" t="s">
+        <v>879</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="8" t="s">
+        <v>881</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="8" t="s">
+        <v>883</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="8" t="s">
+        <v>885</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="8" t="s">
+        <v>887</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="8" t="s">
+        <v>889</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="8" t="s">
+        <v>891</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="8" t="s">
+        <v>893</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="8" t="s">
+        <v>895</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="8" t="s">
+        <v>897</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="8" t="s">
+        <v>899</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="8" t="s">
+        <v>901</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="8" t="s">
+        <v>903</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="8" t="s">
+        <v>905</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="8" t="s">
+        <v>907</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="8" t="s">
+        <v>909</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="8" t="s">
+        <v>911</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="8" t="s">
+        <v>913</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="8" t="s">
+        <v>915</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="8" t="s">
+        <v>917</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="8" t="s">
+        <v>919</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="8" t="s">
+        <v>923</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="8" t="s">
+        <v>925</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="8" t="s">
+        <v>927</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="8" t="s">
+        <v>929</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="8" t="s">
+        <v>931</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="8" t="s">
+        <v>933</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="8" t="s">
+        <v>935</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="8" t="s">
+        <v>937</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="8" t="s">
+        <v>939</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="8" t="s">
+        <v>941</v>
+      </c>
+      <c r="B81" s="8" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="8" t="s">
+        <v>943</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="8" t="s">
+        <v>945</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="8" t="s">
+        <v>947</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="8" t="s">
+        <v>949</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="8" t="s">
+        <v>951</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="8" t="s">
+        <v>953</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="8" t="s">
+        <v>957</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="8" t="s">
+        <v>959</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="8" t="s">
+        <v>961</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="8" t="s">
+        <v>963</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="8" t="s">
+        <v>965</v>
+      </c>
+      <c r="B93" s="8" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="8" t="s">
+        <v>967</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="8" t="s">
+        <v>969</v>
+      </c>
+      <c r="B95" s="8" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="8" t="s">
+        <v>971</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="8" t="s">
+        <v>973</v>
+      </c>
+      <c r="B97" s="8" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="8" t="s">
+        <v>975</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="8" t="s">
+        <v>977</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="8" t="s">
+        <v>979</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="8" t="s">
+        <v>981</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="8" t="s">
+        <v>983</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="8" t="s">
+        <v>985</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="8" t="s">
+        <v>987</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="8" t="s">
+        <v>989</v>
+      </c>
+      <c r="B105" s="8" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="8" t="s">
+        <v>991</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="8" t="s">
+        <v>993</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="8" t="s">
+        <v>995</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="8" t="s">
+        <v>997</v>
+      </c>
+      <c r="B109" s="8" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="8" t="s">
+        <v>999</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="8" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B111" s="8" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="8" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="8" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="8" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="8" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="8" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="8" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="8" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="8" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="8" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="8" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="8" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="8" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" s="8" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" s="8" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" s="8" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" s="8" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="8" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" s="8" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" s="8" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="8" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="8" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="8" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="8" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="8" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="8" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="8" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="8" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="8" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="8" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="8" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="8" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="8" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="8" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="8" t="s">
+        <v>1073</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="8" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="8" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="8" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="8" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="8" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="8" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="8" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="8" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="8" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="8" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="8" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="8" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="8" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="8" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="8" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="8" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="8" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="8" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="8" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="8" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>1114</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="8" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="8" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="8" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="8" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B171" s="8" t="s">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="8" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B172" s="8" t="s">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="8" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B173" s="8" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="8" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B174" s="8" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="8" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B175" s="8" t="s">
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="8" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B176" s="8" t="s">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="8" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B177" s="8" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="8" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B178" s="8" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="8" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B179" s="8" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="8" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B180" s="8" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="8" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B181" s="8" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="8" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B182" s="8" t="s">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="8" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B183" s="8" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="8" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B184" s="8" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="8" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B185" s="8" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="8" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B186" s="8" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="8" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B187" s="8" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="8" t="s">
+        <v>1155</v>
+      </c>
+      <c r="B188" s="8" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="8" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B189" s="8" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="8" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B190" s="8" t="s">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="8" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B191" s="8" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="8" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B192" s="8" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="8" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B193" s="8" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="8" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B194" s="8" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="8" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B195" s="8" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="8" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B196" s="8" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B197" s="8" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="8" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B198" s="8" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="8" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B199" s="8" t="s">
+        <v>1178</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="8" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B200" s="8" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="8" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B201" s="8" t="s">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="8" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B202" s="8" t="s">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="8" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B203" s="8" t="s">
+        <v>1186</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="8" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B204" s="8" t="s">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="8" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B205" s="8" t="s">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="8" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B206" s="8" t="s">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="8" t="s">
+        <v>1193</v>
+      </c>
+      <c r="B207" s="8" t="s">
+        <v>1194</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="8" t="s">
+        <v>1195</v>
+      </c>
+      <c r="B208" s="8" t="s">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="8" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B209" s="8" t="s">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="8" t="s">
+        <v>1199</v>
+      </c>
+      <c r="B210" s="8" t="s">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="8" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B211" s="8" t="s">
+        <v>1202</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="8" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B212" s="8" t="s">
+        <v>1204</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="8" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B213" s="8" t="s">
+        <v>1206</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="8" t="s">
+        <v>1207</v>
+      </c>
+      <c r="B214" s="8" t="s">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="8" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B215" s="8" t="s">
+        <v>1210</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="8" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B216" s="8" t="s">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="8" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B217" s="8" t="s">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="8" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B218" s="8" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="8" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B219" s="8" t="s">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="8" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B220" s="8" t="s">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="8" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B221" s="8" t="s">
+        <v>1222</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="8" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B222" s="8" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="8" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B223" s="8" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="8" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B224" s="8" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="8" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B225" s="8" t="s">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="8" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B226" s="8" t="s">
+        <v>1232</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="8" t="s">
+        <v>1233</v>
+      </c>
+      <c r="B227" s="8" t="s">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="8" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B228" s="8" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="8" t="s">
+        <v>1236</v>
+      </c>
+      <c r="B229" s="8" t="s">
+        <v>1237</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="8" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B230" s="8" t="s">
+        <v>1239</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="8" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B231" s="8" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="8" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B232" s="8" t="s">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B233" s="8" t="s">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="8" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B234" s="8" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B235" s="8" t="s">
+        <v>1249</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="8" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B236" s="8" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="8" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B237" s="8" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="8" t="s">
+        <v>1254</v>
+      </c>
+      <c r="B238" s="8" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="8" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B239" s="8" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="8" t="s">
+        <v>1258</v>
+      </c>
+      <c r="B240" s="8" t="s">
+        <v>1259</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="8" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B241" s="8" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="8" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B242" s="8" t="s">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="8" t="s">
+        <v>1264</v>
+      </c>
+      <c r="B243" s="8" t="s">
+        <v>1265</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="8" t="s">
+        <v>1266</v>
+      </c>
+      <c r="B244" s="8" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="8" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B245" s="8" t="s">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="8" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B246" s="8" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="8" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B247" s="8" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="8" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B248" s="8" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="8" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B249" s="8" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="8" t="s">
+        <v>1278</v>
+      </c>
+      <c r="B250" s="8" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="8" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B251" s="8" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="8" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B252" s="8" t="s">
+        <v>1283</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="8" t="s">
+        <v>1284</v>
+      </c>
+      <c r="B253" s="8" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="8" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B254" s="8" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="8" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B255" s="8" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="8" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B256" s="8" t="s">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="8" t="s">
+        <v>1292</v>
+      </c>
+      <c r="B257" s="8" t="s">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="8" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B258" s="8" t="s">
+        <v>1295</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="8" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B259" s="8" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="8" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B260" s="8" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="8" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B261" s="8" t="s">
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="8" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B262" s="8" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="8" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B263" s="8" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="8" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B264" s="8" t="s">
+        <v>1307</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B265" s="8" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="8" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B266" s="8" t="s">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="8" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B267" s="8" t="s">
+        <v>1313</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="8" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B268" s="8" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="8" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B269" s="8" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="8" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B270" s="8" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="8" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B271" s="8" t="s">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="8" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B272" s="8" t="s">
+        <v>1322</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -30559,7 +34274,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="5" t="s">
-        <v>781</v>
+        <v>1323</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>90</v>
@@ -30568,88 +34283,88 @@
         <v>508</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>782</v>
+        <v>1324</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>783</v>
+        <v>1325</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>784</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="8" t="s">
-        <v>785</v>
+        <v>1327</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8" t="s">
-        <v>786</v>
+        <v>1328</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>787</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="8" t="s">
-        <v>785</v>
+        <v>1327</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
       <c r="E3" s="8" t="s">
-        <v>788</v>
+        <v>1330</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>789</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="8" t="s">
-        <v>785</v>
+        <v>1327</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="s">
-        <v>790</v>
+        <v>1332</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>791</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="8" t="s">
-        <v>785</v>
+        <v>1327</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
       <c r="E5" s="8" t="s">
-        <v>792</v>
+        <v>1334</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>793</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="8" t="s">
-        <v>785</v>
+        <v>1327</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8" t="s">
-        <v>794</v>
+        <v>1336</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>795</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>180</v>
@@ -30658,18 +34373,18 @@
         <v>609</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>797</v>
+        <v>982</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>798</v>
+        <v>981</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>187</v>
@@ -30678,18 +34393,18 @@
         <v>758</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>800</v>
+        <v>1279</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>801</v>
+        <v>1278</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>208</v>
@@ -30698,18 +34413,18 @@
         <v>610</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>802</v>
+        <v>984</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>803</v>
+        <v>983</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>804</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>216</v>
@@ -30718,18 +34433,18 @@
         <v>765</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>805</v>
+        <v>1293</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>806</v>
+        <v>1292</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>804</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>239</v>
@@ -30738,18 +34453,18 @@
         <v>525</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>808</v>
+        <v>813</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>804</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>224</v>
@@ -30758,18 +34473,18 @@
         <v>599</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>809</v>
+        <v>962</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>810</v>
+        <v>961</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>804</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>261</v>
@@ -30778,18 +34493,18 @@
         <v>513</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>811</v>
+        <v>790</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>812</v>
+        <v>789</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>274</v>
@@ -30798,18 +34513,18 @@
         <v>759</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>813</v>
+        <v>1281</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>814</v>
+        <v>1280</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>287</v>
@@ -30818,18 +34533,18 @@
         <v>601</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>815</v>
+        <v>966</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>816</v>
+        <v>965</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>287</v>
@@ -30838,18 +34553,18 @@
         <v>648</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>817</v>
+        <v>1060</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>818</v>
+        <v>1059</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>363</v>
@@ -30858,18 +34573,18 @@
         <v>588</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>819</v>
+        <v>940</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>820</v>
+        <v>939</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>804</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>377</v>
@@ -30878,18 +34593,18 @@
         <v>563</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>821</v>
+        <v>890</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>822</v>
+        <v>889</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>804</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>417</v>
@@ -30898,18 +34613,18 @@
         <v>665</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>823</v>
+        <v>1094</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>824</v>
+        <v>1093</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B20" s="8" t="s">
         <v>424</v>
@@ -30918,18 +34633,18 @@
         <v>569</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>825</v>
+        <v>902</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>826</v>
+        <v>901</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>437</v>
@@ -30938,18 +34653,18 @@
         <v>724</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>827</v>
+        <v>1212</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>828</v>
+        <v>1211</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>481</v>
@@ -30958,18 +34673,18 @@
         <v>718</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>829</v>
+        <v>1200</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>830</v>
+        <v>1199</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="8" t="s">
-        <v>796</v>
+        <v>1338</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>468</v>
@@ -30978,18 +34693,18 @@
         <v>570</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>831</v>
+        <v>904</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>832</v>
+        <v>903</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>799</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="8" t="s">
-        <v>833</v>
+        <v>1341</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>287</v>
@@ -30998,18 +34713,18 @@
         <v>648</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>817</v>
+        <v>1060</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>818</v>
+        <v>1059</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>834</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="8" t="s">
-        <v>833</v>
+        <v>1341</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>468</v>
@@ -31018,13 +34733,13 @@
         <v>570</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>831</v>
+        <v>904</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>832</v>
+        <v>903</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>835</v>
+        <v>1343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add presenter export list
</commit_message>
<xml_diff>
--- a/exports/WIC2026_Programme_Publish.xlsx
+++ b/exports/WIC2026_Programme_Publish.xlsx
@@ -22,7 +22,7 @@
     <t>World Inequality Conference 2026</t>
   </si>
   <si>
-    <t>Generated: 2026-05-28 17:04</t>
+    <t>Generated: 2026-05-29 15:56</t>
   </si>
   <si>
     <t>This programme covers parallel sessions only. For plenary sessions, see the plenary sessions programme.</t>
@@ -2994,222 +2994,265 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>D1-B3-R2-21 | Accumulation dynamics (1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Returns to wealth for everyone: Long-run evolution of group-specific rates of return along the wealth distribution</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Filip Novokmet</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Saving Rate Heterogeneity across the Wealth (Rank) Distribution in the United States</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Christophe Van Langenhove</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Housing Returns across the Income Distribution</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Natalia Khorunzhina</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>The Extraordinary Rise in the Wealth of Older American Households</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Edward Wolff</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Ideological Shifts and Wealth Dynamics: Unraveling the Century-Long Accumulation of Chinese National Wealth, 1911-2020</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Zhexun Mo (Chair)</t>
+      <t>D1-B3-R2-21 | Global inequalities</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Global South dependence on production in the core: an empirical assessment of trends from 1995-2020</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Omer Tayyab</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Argue, Pledge and Implement: Investigating the Role of Fairness in International Climate Policy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Martino Kuntze</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Domestic Inequality and Global Imbalances</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jan Mazza</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Redressing hyper-globalisation and the inequities systemically generated in GVCs: Multilateral efforts at the UN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Gabriele Koehler</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Unequal Exchange and North-South Relations: Evidence from Global Trade Flows and the World Balance of Payments 1800-2025</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Gaston Nievas (Chair)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measuring Global Inequality: How accounting for inequality within the household affects the global profile</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Samuel Kofi Tetteh-Baah</t>
     </r>
   </si>
   <si>
@@ -8531,265 +8574,222 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>D2-B4-R1-10 | Global inequalities</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Global South dependence on production in the core: an empirical assessment of trends from 1995-2020</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Omer Tayyab</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Argue, Pledge and Implement: Investigating the Role of Fairness in International Climate Policy</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Martino Kuntze</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Domestic Inequality and Global Imbalances</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Jan Mazza</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Redressing hyper-globalisation and the inequities systemically generated in GVCs: Multilateral efforts at the UN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Gabriele Koehler</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Unequal Exchange and North-South Relations: Evidence from Global Trade Flows and the World Balance of Payments 1800-2025</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Gaston Nievas (Chair)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measuring Global Inequality: How accounting for inequality within the household affects the global profile</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Samuel Kofi Tetteh-Baah</t>
+      <t>D2-B4-R1-10 | Accumulation dynamics (1)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Returns to wealth for everyone: Long-run evolution of group-specific rates of return along the wealth distribution</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Filip Novokmet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Saving Rate Heterogeneity across the Wealth (Rank) Distribution in the United States</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Christophe Van Langenhove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Housing Returns across the Income Distribution</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Natalia Khorunzhina</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Extraordinary Rise in the Wealth of Older American Households</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Edward Wolff</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ideological Shifts and Wealth Dynamics: Unraveling the Century-Long Accumulation of Chinese National Wealth, 1911-2020</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Zhexun Mo (Chair)</t>
     </r>
   </si>
   <si>
@@ -13196,7 +13196,7 @@
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
     </row>
-    <row r="13" spans="1:7" ht="262" customHeight="1">
+    <row r="13" spans="1:7" ht="224" customHeight="1">
       <c r="A13" s="6" t="s">
         <v>34</v>
       </c>

</xml_diff>